<commit_message>
Encode compound/nested-set reps, drop active-safety text, document flatten decision
build_library.py now pre-builds the real rep rows for the max-dive simulator,
broken-200, and FRC+sprint exercises (flattened heterogeneous blocks with
set_repeat for the outer repeat, sprints labeled via the rep note), records the
nested-set flatten decision in the docstring, and removes the active-safety
phrase from the simulator goal. Fixtures regenerated and schema-validated.
</commit_message>
<xml_diff>
--- a/docs/exercise-canon-and-mapping.xlsx
+++ b/docs/exercise-canon-and-mapping.xlsx
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>80% PB, short dive, then a max push, with breaths between. Active safety.</t>
+          <t>80% PB, short dive, then a max push, with breaths between.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>80% PB, short dive, then a max push, with breaths between. Active safety.</t>
+          <t>80% PB, short dive, then a max push, with breaths between.</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Split NWU sub-max with movement into its own exercise
STA 2's NWU-with-movement was folded into sta-nwu-submax as a
movement: still|moving cue, so it never appeared in the library list.
It is now sta-nwu-submax-moving (soft 4:6 belly-only HV, constant
movement, full recovery, per the STA note), the STA 2 mapping points
at it, and the base NWU sub-max drops the movement option. Catalog is
45 exercises; the V-shape affinity now pairs with the moving variant.
</commit_message>
<xml_diff>
--- a/docs/exercise-canon-and-mapping.xlsx
+++ b/docs/exercise-canon-and-mapping.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affinities" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Canonical catalog'!$A$1:$G$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Canonical catalog'!$A$1:$G$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mapping (combined)'!$A$1:$K$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Affinities'!$A$1:$D$31</definedName>
   </definedNames>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -534,24 +534,24 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>No warmup; one sub-max hold to read sensations.</t>
+          <t>No warmup; one still sub-max hold to read sensations.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>HV prep (def 5 min 5:5); movement: still|moving (def still); recovery (def full).</t>
+          <t>HV prep (def 5 min 5:5); recovery (def full).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>sta-co2-increasing</t>
+          <t>sta-nwu-submax-moving</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>CO2 table, increasing holds</t>
+          <t>NWU sub-max with movement</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -566,29 +566,29 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>co2</t>
+          <t>mental, co2, o2_hypoxia</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Fixed recovery breaths; holds increase from a start, until failure.</t>
+          <t>No warmup; one sub-max hold with constant movement (paddle hands, move arms, never still).</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>recovery breaths (def 5); start (def 2:00); step (def +20-30s); termination (def until failure).</t>
+          <t>HV prep (def 5 min soft 4:6, belly only); recovery (def full).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>sta-co2-vshape</t>
+          <t>sta-co2-increasing</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>CO2 table, V-shaped</t>
+          <t>CO2 table, increasing holds</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -608,24 +608,24 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Holds descend toward ~1 min then ascend; maximize total time under discomfort.</t>
+          <t>Fixed recovery breaths; holds increase from a start, until failure.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>recovery breaths (def 2); start (def ~50% PB); HV prep (def 4:6 soft).</t>
+          <t>recovery breaths (def 5); start (def 2:00); step (def +20-30s); termination (def until failure).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>sta-co2-1breath</t>
+          <t>sta-co2-vshape</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1-breath CO2 ladder</t>
+          <t>CO2 table, V-shaped</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -645,24 +645,24 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1-breath recovery; short repeated holds until quality drops.</t>
+          <t>Holds descend toward ~1 min then ascend; maximize total time under discomfort.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>ladder mode: absolute|1C+X (def 1C+X); step (def +10s); termination (def quality-drop).</t>
+          <t>recovery breaths (def 2); start (def ~50% PB); HV prep (def 4:6 soft).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>sta-co2-short-intense</t>
+          <t>sta-co2-1breath</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Short &amp; intense CO2</t>
+          <t>1-breath CO2 ladder</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -682,24 +682,24 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>5-6 FL holds at a sustainable duration, 2-breath recovery only.</t>
+          <t>1-breath recovery; short repeated holds until quality drops.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>n holds (def 6); hold (def sustainable, e.g. 2:30); recovery (def 2 breaths).</t>
+          <t>ladder mode: absolute|1C+X (def 1C+X); step (def +10s); termination (def quality-drop).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>sta-co2-decreasing-rec</t>
+          <t>sta-co2-short-intense</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Medium &amp; moderate CO2</t>
+          <t>Short &amp; intense CO2</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -714,29 +714,29 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>co2, mental</t>
+          <t>co2</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Fixed hold; recovery shrinks each rep.</t>
+          <t>5-6 FL holds at a sustainable duration, 2-breath recovery only.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>hold (def sized to contraction duration); recovery start (def 60s); step (def -10s).</t>
+          <t>n holds (def 6); hold (def sustainable, e.g. 2:30); recovery (def 2 breaths).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>sta-co2-square</t>
+          <t>sta-co2-decreasing-rec</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Soft &amp; medium CO2 (square breathing)</t>
+          <t>Medium &amp; moderate CO2</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -751,29 +751,29 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>mental, co2</t>
+          <t>co2, mental</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Square breathing held for a long duration.</t>
+          <t>Fixed hold; recovery shrinks each rep.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>box length (def 10s); duration (def 30 min).</t>
+          <t>hold (def sized to contraction duration); recovery start (def 60s); step (def -10s).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>sta-co2-second-hold</t>
+          <t>sta-co2-square</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>CO2, challenging second hold</t>
+          <t>Soft &amp; medium CO2 (square breathing)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -788,29 +788,29 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>co2</t>
+          <t>mental, co2</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Sub-max, a few recovery breaths, then a max-effort second hold as the target.</t>
+          <t>Square breathing held for a long duration.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>first hold (def ~70% PB); recovery breaths (def 3); prep (def 5 min 5:5).</t>
+          <t>box length (def 10s); duration (def 30 min).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>sta-get-high</t>
+          <t>sta-co2-second-hold</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Get high (oxygen table)</t>
+          <t>CO2, challenging second hold</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -825,29 +825,29 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>o2_hypoxia</t>
+          <t>co2</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Strong HV prep before each; add 1 min per hold until it gets hard, then add 30s only.</t>
+          <t>Sub-max, a few recovery breaths, then a max-effort second hold as the target.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>HV pattern (def 2:2 strong); start hold (def 1 min); step (def +1 min, then +30s once hard).</t>
+          <t>first hold (def ~70% PB); recovery breaths (def 3); prep (def 5 min 5:5).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>sta-el</t>
+          <t>sta-get-high</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Empty-lung set</t>
+          <t>Get high (oxygen table)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -857,34 +857,34 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>main, warmup</t>
+          <t>main</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>o2_hypoxia, mental</t>
+          <t>o2_hypoxia</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>RV/EL holds, increasing duration.</t>
+          <t>Strong HV prep before each; add 1 min per hold until it gets hard, then add 30s only.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>n (def 5); style: relaxed-belly|pull-and-release (def relaxed-belly); recovery (def 2-3 min).</t>
+          <t>HV pattern (def 2:2 strong); start hold (def 1 min); step (def +1 min, then +30s once hard).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>sta-el-fl-switch</t>
+          <t>sta-el</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>EL/FL switch</t>
+          <t>Empty-lung set</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -904,24 +904,24 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Alternating EL and FL holds, both increasing.</t>
+          <t>RV/EL holds, increasing duration.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>EL step (def +20s); FL step (def +20-30s); recovery (def 2 min 4:6 HV); as-warmup: stay below PB margins.</t>
+          <t>n (def 5); style: relaxed-belly|pull-and-release (def relaxed-belly); recovery (def 2-3 min).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>sta-1c-plus</t>
+          <t>sta-el-fl-switch</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>First-contraction-plus ladder</t>
+          <t>EL/FL switch</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -931,34 +931,34 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>main, warmup</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>co2, mental</t>
+          <t>o2_hypoxia, mental</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Increasing breathing prep; hold target = 1C + Xs across reps.</t>
+          <t>Alternating EL and FL holds, both increasing.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>prep ramp (def 2-&gt;4 min); 1C+X schedule (def +0/20/40/60/80s); recovery mode (def increasing prep|fixed 2 min).</t>
+          <t>EL step (def +20s); FL step (def +20-30s); recovery (def 2 min 4:6 HV); as-warmup: stay below PB margins.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>sta-frc-awareness</t>
+          <t>sta-1c-plus</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>FRC CO2 awareness</t>
+          <t>First-contraction-plus ladder</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -973,29 +973,29 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>co2</t>
+          <t>co2, mental</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>FL then exhale to FRC then a short hold; short recovery only.</t>
+          <t>Increasing breathing prep; hold target = 1C + Xs across reps.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>hold steps (def 15/30/45s); recovery (def 1 min).</t>
+          <t>prep ramp (def 2-&gt;4 min); 1C+X schedule (def +0/20/40/60/80s); recovery mode (def increasing prep|fixed 2 min).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>sta-high-volume</t>
+          <t>sta-frc-awareness</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>High-volume holds</t>
+          <t>FRC CO2 awareness</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1010,29 +1010,29 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>volume, co2, o2_hypoxia</t>
+          <t>co2</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Repeat a % of PB many times.</t>
+          <t>FL then exhale to FRC then a short hold; short recovery only.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>% PB (def 70); n reps (def 3-10); rest (def long/unlimited); reduce-prep-each-rep (def off).</t>
+          <t>hold steps (def 15/30/45s); recovery (def 1 min).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>sta-progressive-fl</t>
+          <t>sta-high-volume</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Progressive FL to max</t>
+          <t>High-volume holds</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1047,29 +1047,29 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>co2, mental</t>
+          <t>volume, co2, o2_hypoxia</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Comfortable -&gt; strong sub-max -&gt; max(-ish) FL for the day.</t>
+          <t>Repeat a % of PB many times.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>prep (def 5 min); sequence (def 3 holds).</t>
+          <t>% PB (def 70); n reps (def 3-10); rest (def long/unlimited); reduce-prep-each-rep (def off).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>sta-max</t>
+          <t>sta-progressive-fl</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>STA max attempt</t>
+          <t>Progressive FL to max</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1084,29 +1084,29 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>performance</t>
+          <t>co2, mental</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Single maximal breath-hold. The performance test warm-ups are compared against.</t>
+          <t>Comfortable -&gt; strong sub-max -&gt; max(-ish) FL for the day.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>HV prep (def 5 min 5:5); lung (def FL).</t>
+          <t>prep (def 5 min); sequence (def 3 holds).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>sta-cooldown-easy</t>
+          <t>sta-max</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Easy cool-down STA</t>
+          <t>STA max attempt</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1116,34 +1116,34 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>cooldown</t>
+          <t>main</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>mental</t>
+          <t>performance</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Light, relaxed sub-max hold to finish on something easy.</t>
+          <t>Single maximal breath-hold. The performance test warm-ups are compared against.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>hold (def light submax); recovery (def full).</t>
+          <t>HV prep (def 5 min 5:5); lung (def FL).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>sta-wu-fl-progression</t>
+          <t>sta-cooldown-easy</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>WU: FL progression</t>
+          <t>Easy cool-down STA</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1153,34 +1153,34 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>warmup</t>
+          <t>cooldown</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>co2, mental</t>
+          <t>mental</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>1C+20 / 1C+40 / 1C+60 FL holds.</t>
+          <t>Light, relaxed sub-max hold to finish on something easy.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>steps (def 1C+20/40/60); recovery (def 3 min).</t>
+          <t>hold (def light submax); recovery (def full).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>sta-wu-frc-progression</t>
+          <t>sta-wu-fl-progression</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>WU: FRC progression</t>
+          <t>WU: FL progression</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1195,29 +1195,29 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>co2</t>
+          <t>co2, mental</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>FRC holds through the first hard contractions (not to hypoxia).</t>
+          <t>1C+20 / 1C+40 / 1C+60 FL holds.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>n (def 3); recovery (def 3-4 min).</t>
+          <t>steps (def 1C+20/40/60); recovery (def 3 min).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>sta-wu-contraction-delay</t>
+          <t>sta-wu-frc-progression</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>WU: contraction delay</t>
+          <t>WU: FRC progression</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1232,29 +1232,29 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>co2, mental</t>
+          <t>co2</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Repeat holds until 1C arrives at the right time, then go for max.</t>
+          <t>FRC holds through the first hard contractions (not to hypoxia).</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>trigger (def 1C timing feels right).</t>
+          <t>n (def 3); recovery (def 3-4 min).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>sta-wu-rv-fl</t>
+          <t>sta-wu-contraction-delay</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>WU: RV progression + 1 FL</t>
+          <t>WU: contraction delay</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1269,29 +1269,29 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>o2_hypoxia, co2</t>
+          <t>co2, mental</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>3 RV holds (easy/moderate/hard) + 1 FL.</t>
+          <t>Repeat holds until 1C arrives at the right time, then go for max.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>FL target (def ~1.5 min under PB).</t>
+          <t>trigger (def 1C timing feels right).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>sta-wu-nwu-hard-start</t>
+          <t>sta-wu-rv-fl</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>WU: NWU hard start</t>
+          <t>WU: RV progression + 1 FL</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1306,29 +1306,29 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>co2, o2_hypoxia</t>
+          <t>o2_hypoxia, co2</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>One hard FL near PB-1min, recover, then max.</t>
+          <t>3 RV holds (easy/moderate/hard) + 1 FL.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>hard hold (def PB-1 min); recovery (def 5 min + strong HV).</t>
+          <t>FL target (def ~1.5 min under PB).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>sta-wu-3rv-3fl</t>
+          <t>sta-wu-nwu-hard-start</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>WU: 3xRV + 3xFL</t>
+          <t>WU: NWU hard start</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1343,66 +1343,66 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>o2_hypoxia</t>
+          <t>co2, o2_hypoxia</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>3 EL holds then 3 FL holds.</t>
+          <t>One hard FL near PB-1min, recover, then max.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>RV recovery (def 3 min); FL recovery (def 5 min).</t>
+          <t>hard hold (def PB-1 min); recovery (def 5 min + strong HV).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>dyn-nwu-submax</t>
+          <t>sta-wu-3rv-3fl</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>NWU sub-max (dynamic)</t>
+          <t>WU: 3xRV + 3xFL</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>warmup</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>mental, o2_hypoxia</t>
+          <t>o2_hypoxia</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>~70-80% feel, explore sensations, no fixed distance.</t>
+          <t>3 EL holds then 3 FL holds.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>% feel (def 70-80); variant: plain|to-1C+contractions (def plain); discipline (def any; DNF shorter).</t>
+          <t>RV recovery (def 3 min); FL recovery (def 5 min).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>dyn-max</t>
+          <t>dyn-nwu-submax</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Dynamic max attempt</t>
+          <t>NWU sub-max (dynamic)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1417,29 +1417,29 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>performance</t>
+          <t>mental, o2_hypoxia</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Single maximal distance attempt. The performance test warm-ups are compared against.</t>
+          <t>~70-80% feel, explore sensations, no fixed distance.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>discipline (def any; DNF shorter).</t>
+          <t>% feel (def 70-80); variant: plain|to-1C+contractions (def plain); discipline (def any; DNF shorter).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>dyn-max-simulator</t>
+          <t>dyn-max</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Max dive simulator</t>
+          <t>Dynamic max attempt</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1454,29 +1454,29 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>o2_hypoxia</t>
+          <t>performance</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>80% PB, short dive, then a max push, with breaths between.</t>
+          <t>Single maximal distance attempt. The performance test warm-ups are compared against.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>% PB (def 80); short leg (def min{60m,30% PB}); RB (def 2 then 3).</t>
+          <t>discipline (def any; DNF shorter).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>dyn-volume-fixed</t>
+          <t>dyn-max-simulator</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Volume: fixed reps</t>
+          <t>Max dive simulator</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1491,29 +1491,29 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>volume, co2</t>
+          <t>o2_hypoxia</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>N x a fixed distance with a set recovery (NOT goal-maximize).</t>
+          <t>80% PB, short dive, then a max push, with breaths between.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>n reps; distance (def 50/75m; shorter for DNF); recovery; pacing (def even).</t>
+          <t>% PB (def 80); short leg (def min{60m,30% PB}); RB (def 2 then 3).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>dyn-volume-maximize</t>
+          <t>dyn-volume-fixed</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Volume: maximize total distance</t>
+          <t>Volume: fixed reps</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1528,34 +1528,34 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>volume, o2_hypoxia</t>
+          <t>volume, co2</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>N dives where the goal is maximizing total distance; distance not fixed.</t>
+          <t>N x a fixed distance with a set recovery (NOT goal-maximize).</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>n dives; recovery (often shrinks across session).</t>
+          <t>n reps; distance (def 50/75m; shorter for DNF); recovery; pacing (def even).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>dyn-volume-technique</t>
+          <t>dyn-volume-maximize</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Volume: technique drill</t>
+          <t>Volume: maximize total distance</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>DNF</t>
+          <t>any</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1565,34 +1565,34 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>technique, co2</t>
+          <t>volume, o2_hypoxia</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Sets alternating legs-only and normal (or arms-only), minimal recovery.</t>
+          <t>N dives where the goal is maximizing total distance; distance not fixed.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>n sets (def 8-10); block (def 50m legs-only + 50m normal); recovery (def minimal).</t>
+          <t>n dives; recovery (often shrinks across session).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>dyn-pyramid</t>
+          <t>dyn-volume-technique</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Pyramid drills</t>
+          <t>Volume: technique drill</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>DNF</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1602,29 +1602,29 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>co2, volume</t>
+          <t>technique, co2</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>25-50-75-50-25; minimal-but-confident recovery; full recovery between sets.</t>
+          <t>Sets alternating legs-only and normal (or arms-only), minimal recovery.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>ladder (def 25-50-75-50-25); recovery (def minimal/confident); n pyramids (user adds as many as wanted); distances shorter for DNF.</t>
+          <t>n sets (def 8-10); block (def 50m legs-only + 50m normal); recovery (def minimal).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>dyn-inverse-pyramid</t>
+          <t>dyn-pyramid</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Inverse pyramid</t>
+          <t>Pyramid drills</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1644,24 +1644,24 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>75-50-25-50-75; minimal-but-confident recovery.</t>
+          <t>25-50-75-50-25; minimal-but-confident recovery; full recovery between sets.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>ladder (def 75-50-25-50-75); recovery (def &lt; swim time, cap 90s); sets (def 2).</t>
+          <t>ladder (def 25-50-75-50-25); recovery (def minimal/confident); n pyramids (user adds as many as wanted); distances shorter for DNF.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>dyn-descending</t>
+          <t>dyn-inverse-pyramid</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Descending distance</t>
+          <t>Inverse pyramid</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1676,29 +1676,29 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>co2</t>
+          <t>co2, volume</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Long doable distance, then ~20% less, then ~20% less again.</t>
+          <t>75-50-25-50-75; minimal-but-confident recovery.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>start (def long doable); step (def -20%); n (def 3); recovery (def minimal).</t>
+          <t>ladder (def 75-50-25-50-75); recovery (def &lt; swim time, cap 90s); sets (def 2).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>dyn-sweet16</t>
+          <t>dyn-descending</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Sweet 16</t>
+          <t>Descending distance</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1713,29 +1713,29 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>co2, technique</t>
+          <t>co2</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>16 x 25m as quickly as possible.</t>
+          <t>Long doable distance, then ~20% less, then ~20% less again.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>reps (def 16); distance (def 25m); recovery (def 0-30s).</t>
+          <t>start (def long doable); step (def -20%); n (def 3); recovery (def minimal).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>dyn-sprints</t>
+          <t>dyn-sweet16</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Sprint set</t>
+          <t>Sweet 16</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1750,29 +1750,29 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>fitness_lactic, technique</t>
+          <t>co2, technique</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Max sprints with short recovery.</t>
+          <t>16 x 25m as quickly as possible.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>distance (def 25/50m); n; recovery (short).</t>
+          <t>reps (def 16); distance (def 25m); recovery (def 0-30s).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>dyn-frc-sprint</t>
+          <t>dyn-sprints</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>FRC dive + sprints</t>
+          <t>Sprint set</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1787,29 +1787,29 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>fitness_lactic</t>
+          <t>fitness_lactic, technique</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>FRC dive (longest possible) then a max-sprint ladder.</t>
+          <t>Max sprints with short recovery.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>FRC distance (def 50-100m); sprint ladder (def 3x25m, growing recovery); sets (def 3).</t>
+          <t>distance (def 25/50m); n; recovery (short).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>dyn-elastic-sprint-max</t>
+          <t>dyn-frc-sprint</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Elastic sprints into max</t>
+          <t>FRC dive + sprints</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1829,24 +1829,24 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Elastic-band max sprints then straight into a max dive.</t>
+          <t>FRC dive (longest possible) then a max-sprint ladder.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>sprints (def 4 x 15s, 15s rest); sets (def 2).</t>
+          <t>FRC distance (def 50-100m); sprint ladder (def 3x25m, growing recovery); sets (def 3).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>dyn-stop-start</t>
+          <t>dyn-elastic-sprint-max</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Stop-start (STA then swim)</t>
+          <t>Elastic sprints into max</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1861,29 +1861,29 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>mental, co2</t>
+          <t>fitness_lactic</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>A STA hold, then straight into a dynamic swim.</t>
+          <t>Elastic-band max sprints then straight into a max dive.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>STA duration (def 1:30); then distance/sub-max.</t>
+          <t>sprints (def 4 x 15s, 15s rest); sets (def 2).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>dyn-start-stop</t>
+          <t>dyn-stop-start</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Start-stop (swim then STA)</t>
+          <t>Stop-start (STA then swim)</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1903,24 +1903,24 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>A dynamic swim, then straight into a STA hold. (Not in the library; added.)</t>
+          <t>A STA hold, then straight into a dynamic swim.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>distance; then STA duration.</t>
+          <t>STA duration (def 1:30); then distance/sub-max.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>dyn-stop-dyn</t>
+          <t>dyn-start-stop</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Stop in the middle (dive-STA-dive)</t>
+          <t>Start-stop (swim then STA)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1940,24 +1940,24 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>A dynamic, then a STA hold, then another dynamic. (Not in the library; added.)</t>
+          <t>A dynamic swim, then straight into a STA hold. (Not in the library; added.)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>leg-1 distance; STA duration; leg-2 distance.</t>
+          <t>distance; then STA duration.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>dyn-transition-ladder</t>
+          <t>dyn-stop-dyn</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>STA-to-dynamic transition ladder</t>
+          <t>Stop in the middle (dive-STA-dive)</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -1977,29 +1977,29 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2-3x STA to 1C/UTB then a dynamic, swimming further each dive.</t>
+          <t>A dynamic, then a STA hold, then another dynamic. (Not in the library; added.)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>mode: FL|crawl|FRC; n per mode (def 2-3).</t>
+          <t>leg-1 distance; STA duration; leg-2 distance.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>dyn-technique</t>
+          <t>dyn-transition-ladder</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Technique drills</t>
+          <t>STA-to-dynamic transition ladder</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>DNF</t>
+          <t>any</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2009,34 +2009,34 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>technique</t>
+          <t>mental, co2</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Arms-only / legs-only / normal, counting strokes to reduce them.</t>
+          <t>2-3x STA to 1C/UTB then a dynamic, swimming further each dive.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>blocks (def 4x each); count (strokes).</t>
+          <t>mode: FL|crawl|FRC; n per mode (def 2-3).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>dyn-tortuga</t>
+          <t>dyn-technique</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Tortuga (slow crawl)</t>
+          <t>Technique drills</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>tortuga</t>
+          <t>DNF</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2046,34 +2046,34 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>mental, co2</t>
+          <t>technique</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Its own discipline. Cover a short distance in the longest possible time; max time, distance irrelevant.</t>
+          <t>Arms-only / legs-only / normal, counting strokes to reduce them.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>distance cap (def 50m).</t>
+          <t>blocks (def 4x each); count (strokes).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>dyn-broken-200</t>
+          <t>dyn-tortuga</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Broken 200m</t>
+          <t>Tortuga (slow crawl)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>tortuga</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2083,59 +2083,96 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>co2</t>
+          <t>mental, co2</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>75m, 50m, 3x25m with minimum recovery; consistent pace.</t>
+          <t>Its own discipline. Cover a short distance in the longest possible time; max time, distance irrelevant.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>structure (def 75/50/3x25); recovery (def minimum, caps 60s/30s/few breaths).</t>
+          <t>distance cap (def 50m).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>dyn-broken-200</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Broken 200m</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>co2</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>75m, 50m, 3x25m with minimum recovery; consistent pace.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>structure (def 75/50/3x25); recovery (def minimum, caps 60s/30s/few breaths).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>dyn-hypercapnic</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Hypercapnic cool-down</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>any</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>cooldown</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>co2, volume</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Continuous swim, breathing every several strokes, no stopping.</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>distance (def 300-500m); breathe every (def 7+ strokes).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G45"/>
+  <autoFilter ref="A1:G46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2267,12 +2304,12 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>No warmup; one sub-max hold to read sensations.</t>
+          <t>No warmup; one still sub-max hold to read sensations.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>5 min strong HV (5:5); movement=still; full recovery</t>
+          <t>5 min strong HV (5:5); full recovery</t>
         </is>
       </c>
     </row>
@@ -2356,12 +2393,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>sta-nwu-submax</t>
+          <t>sta-nwu-submax-moving</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>NWU sub-max</t>
+          <t>NWU sub-max with movement</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -2381,12 +2418,12 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>No warmup; one sub-max hold to read sensations.</t>
+          <t>No warmup; one sub-max hold with constant movement (paddle hands, move arms, never still).</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>soft HV (4:6); movement=moving</t>
+          <t>5 min soft HV (4:6, belly only); full recovery</t>
         </is>
       </c>
     </row>
@@ -7102,7 +7139,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>sta-nwu-submax</t>
+          <t>sta-nwu-submax-moving</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">

</xml_diff>

<commit_message>
Rename CO2 RB tables: 5 x RB increasing, 1 x RB wonka, 2 x RB repeats
</commit_message>
<xml_diff>
--- a/docs/exercise-canon-and-mapping.xlsx
+++ b/docs/exercise-canon-and-mapping.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>CO2 increasing</t>
+          <t>CO2 5 x RB increasing</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CO2 1RB wonka</t>
+          <t>CO2 1 x RB wonka</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>CO2 2RB repeats</t>
+          <t>CO2 2 x RB repeats</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>CO2 increasing</t>
+          <t>CO2 5 x RB increasing</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>CO2 1RB wonka</t>
+          <t>CO2 1 x RB wonka</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>CO2 2RB repeats</t>
+          <t>CO2 2 x RB repeats</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -3880,7 +3880,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>CO2 1RB wonka</t>
+          <t>CO2 1 x RB wonka</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Rename max attempts, pyramids, sprints; refine review-doc metric notes
</commit_message>
<xml_diff>
--- a/docs/exercise-canon-and-mapping.xlsx
+++ b/docs/exercise-canon-and-mapping.xlsx
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>STA max attempt</t>
+          <t>Max attempt: STA</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Dynamic max attempt</t>
+          <t>Max attempt: dynamic</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Pyramid drills</t>
+          <t>Pyramid</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Inverse pyramid</t>
+          <t>Pyramid (inverse)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Sprint set</t>
+          <t>Sprints</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -4792,7 +4792,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Pyramid drills</t>
+          <t>Pyramid</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Sprint set</t>
+          <t>Sprints</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -5248,7 +5248,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Inverse pyramid</t>
+          <t>Pyramid (inverse)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Sprint set</t>
+          <t>Sprints</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Sprint set</t>
+          <t>Sprints</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Inverse pyramid</t>
+          <t>Pyramid (inverse)</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -5932,7 +5932,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Sprint set</t>
+          <t>Sprints</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Sprint set</t>
+          <t>Sprints</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Remove STA-to-dynamic transition ladder; remap DYN 4 to stop-start
</commit_message>
<xml_diff>
--- a/docs/exercise-canon-and-mapping.xlsx
+++ b/docs/exercise-canon-and-mapping.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affinities" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Canonical catalog'!$A$1:$G$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Canonical catalog'!$A$1:$G$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mapping (combined)'!$A$1:$K$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Affinities'!$A$1:$D$31</definedName>
   </definedNames>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1989,17 +1989,17 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>dyn-transition-ladder</t>
+          <t>dyn-technique</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>STA-to-dynamic transition ladder</t>
+          <t>Technique drills</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>DNF</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2009,34 +2009,34 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>mental, co2</t>
+          <t>technique</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2-3x STA to 1C/UTB then a dynamic, swimming further each dive.</t>
+          <t>Arms-only / legs-only / normal, counting strokes to reduce them.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>mode: FL|crawl|FRC; n per mode (def 2-3).</t>
+          <t>blocks (def 4x each); count (strokes).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>dyn-technique</t>
+          <t>dyn-tortuga</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Technique drills</t>
+          <t>Tortuga (slow crawl)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>DNF</t>
+          <t>tortuga</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2046,34 +2046,34 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>technique</t>
+          <t>mental, co2</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Arms-only / legs-only / normal, counting strokes to reduce them.</t>
+          <t>Its own discipline. Cover a short distance in the longest possible time; max time, distance irrelevant.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>blocks (def 4x each); count (strokes).</t>
+          <t>distance cap (def 50m).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>dyn-tortuga</t>
+          <t>dyn-broken-200</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Tortuga (slow crawl)</t>
+          <t>Broken 200m</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>tortuga</t>
+          <t>any</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2083,29 +2083,29 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>mental, co2</t>
+          <t>co2</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Its own discipline. Cover a short distance in the longest possible time; max time, distance irrelevant.</t>
+          <t>75m, 50m, 3x25m with minimum recovery; consistent pace.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>distance cap (def 50m).</t>
+          <t>structure (def 75/50/3x25); recovery (def minimum, caps 60s/30s/few breaths).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>dyn-broken-200</t>
+          <t>dyn-hypercapnic</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Broken 200m</t>
+          <t>Hypercapnic cool-down</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2115,64 +2115,27 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>cooldown</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>co2</t>
+          <t>co2, volume</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>75m, 50m, 3x25m with minimum recovery; consistent pace.</t>
+          <t>Continuous swim, breathing every several strokes, no stopping.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>structure (def 75/50/3x25); recovery (def minimum, caps 60s/30s/few breaths).</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>dyn-hypercapnic</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Hypercapnic cool-down</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>any</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>cooldown</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>co2, volume</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Continuous swim, breathing every several strokes, no stopping.</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
           <t>distance (def 300-500m); breathe every (def 7+ strokes).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G46"/>
+  <autoFilter ref="A1:G45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4502,12 +4465,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>dyn-transition-ladder</t>
+          <t>dyn-stop-start</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>STA-to-dynamic transition ladder</t>
+          <t>Stop-start (STA then swim)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -4527,12 +4490,12 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>2-3x STA to 1C/UTB then a dynamic, swimming further each dive.</t>
+          <t>A STA hold, then straight into a dynamic swim.</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>2-3x STA to 1C/UTB then FL/crawl/FRC, further each dive</t>
+          <t>2-3x STA to 1C/UTB then FL/crawl/FRC, further each dive (was a transition-ladder exercise; folded into stop-start)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate the exercise workbook with the Seals catalog sheet; import order tidy in build_library.py
</commit_message>
<xml_diff>
--- a/docs/exercise-canon-and-mapping.xlsx
+++ b/docs/exercise-canon-and-mapping.xlsx
@@ -10,11 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical catalog" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping (combined)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affinities" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seals catalog" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Canonical catalog'!$A$1:$G$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mapping (combined)'!$A$1:$K$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Affinities'!$A$1:$D$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Seals catalog'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7198,4 +7200,431 @@
   <autoFilter ref="A1:D31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Discipline</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Capacity focus</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Structure</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Editable options (defaults)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>seals-fixed-rest</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Fixed-rest set</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DYNb</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>co2</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Repeated 50 m at your normal dive pace with a rest cap. Base: 4, 5, 6, 7 reps across the four weeks, cap 60 s. Specialization: 6 reps, cap 45 s. Taper: 5 then 4 reps, cap 45 s.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>reps (def 4); distance (def 50m, 25m for newer members); rest cap (def 60s).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>seals-pyramid</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Pyramid</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>DYNb</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>co2</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>50-25-25-50 in weeks 1-2, 50-50-25-50-50 in weeks 3-4, rest no longer than 60 s and shorter when you can.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>ladder (def 50-25-25-50); rest cap (def 60s).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>seals-hypercapnic-swim</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Hypercapnic surface swim</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>swim</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>co2</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Freestyle on the surface in short fins, no wetsuit, breathing a fixed 3 times per 25 m, no stopping. Base 100 to 250 m, build 300 to 350 m, specialization 400 m, taper 300 then 200 m.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>distance (def 100m); breaths per 25m (def 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>seals-recovery-swim</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Recovery swim</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>swim</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>cooldown</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>100 m any style, relaxed, breathing normally, to close every session.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>distance (def 100m).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>seals-over-under</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Over-under warm-up</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>DYNb</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>warmup</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>technique</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>25 m freestyle on the surface, turn, 25 m DYNb underwater without stopping; twice for 100 m.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>rounds (def 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>seals-sprints</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Sprints</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>DYNb</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>fitness_lactic</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>All-out DYNb sprints. Base: 2 sets of 6 x 25 m, 20 s between reps, 2 min between sets (weeks 1-2), then 6 x 50 m with 60 s (weeks 3-4). Build: 5-6 x 75 m with 75-120 s.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>distance (def 25m); reps (def 6); sets (def 2); rest (def 20s); rest between sets (def 2 min).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>seals-dolphin-sprints</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Dolphin sprints</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>DYNb</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>fitness_lactic</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Each rep is 25 m of all-out dolphin kick on the surface (snorkel, or on your back so you can breathe), then a duck dive straight into 10 m underwater at sprint pace. 2 sets of 4 (weeks 5-6), 2 sets of 5 (weeks 7-8), 60-90 s between reps, 3 min between sets, short fins, no wetsuit.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>reps (def 4); sets (def 2); rest (def 90s); rest between sets (def 3 min).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>seals-submax</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Submax dive</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>DYNb</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>o2_hypoxia, mental</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>One dive, no warm-up, no breathe-up, breathing normally beforehand, face dry until you go. Aim for at least the target percentage of your PB with no upper limit, but surface before your limit and never finish shaky. Build 65%, specialization 70-75%, taper 80%.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>% of PB (def 65).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>seals-endurance-ladder</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Endurance ladder</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>DYNb</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>co2, volume</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Mixed 75 m and 50 m with rest no longer than the dive time. Week 9: 1 x 75 + 5 x 50, then convert one 50 into a 75 each week (2 + 4, 3 + 3, 4 + 2).</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>75s (def 1); 50s (def 5); rest (def at most the dive time).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>seals-tortuga</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Tortuga (slow crawl)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>tortuga</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>mental, co2</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Crawl along the bottom as slowly as you can, covering at most 50 m in the longest possible time; no goggles so you do not watch the clock. From week 5, one slow crawl after the sprints, every week.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>distance cap (def 50m).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>